<commit_message>
Cambios en PipelineExecution para admitir subida de archivos junto con popup visual
</commit_message>
<xml_diff>
--- a/data/database/pipelines.xlsx
+++ b/data/database/pipelines.xlsx
@@ -544,7 +544,11 @@
           <t>PDF</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-02-04 13:20:30</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
correcciones en workflows y pipelines
</commit_message>
<xml_diff>
--- a/data/database/pipelines.xlsx
+++ b/data/database/pipelines.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,15 +446,25 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>jsonb</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>input</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>output</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>last_run</t>
         </is>
@@ -476,15 +486,82 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>InitRun -&gt; LoadConfig -&gt; DiscoverInputs -&gt; RunExcelETL -&gt; EnrichWithContext -&gt; ExportConsolidatedExcel</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>{
+    "workflow_metadata": {
+        "name": "SIMCE Lenguaje",
+        "description": "Workflow SIMCE",
+        "input": "EXCEL",
+        "output": "PDF"
+    },
+    "context": {
+        "base_dir": "tests"
+    },
+    "pipeline": [
+        {
+            "step": "InitRun",
+            "params": {
+                "inputs_dir": "tests/input_test/inputs/Lenguaje/inputs"
+            }
+        },
+        {
+            "step": "LoadConfig",
+            "params": {
+                "config_path": "./tests/config_dir/simce_estudiantes_lenguaje.json"
+            }
+        },
+        {
+            "step": "DiscoverInputs",
+            "params": {
+                "rules": {
+                    "estudiantes": {
+                        "extension": ".xlsx",
+                        "contains": "Resultados"
+                    },
+                    "preguntas": {
+                        "extension": ".xlsx",
+                        "contains": "ReportePregunta"
+                    },
+                    "habilidades": {
+                        "extension": ".xlsx",
+                        "contains": "habilidades"
+                    }
+                }
+            }
+        },
+        {
+            "step": "RunExcelETL",
+            "params": {
+                "input_key": "estudiantes"
+            }
+        },
+        {
+            "step": "EnrichWithContext",
+            "params": {}
+        },
+        {
+            "step": "ExportConsolidatedExcel",
+            "params": {}
+        }
+    ]
+}</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>EXCEL</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>PDF</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>2026-01-31 13:28:43</t>
         </is>
@@ -504,17 +581,39 @@
           <t>Diagnóstico Integral de Aprendizaje</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>{
+    "workflow_metadata": {
+        "name": "DIA Extraer respuestas correctas",
+        "description": "Diagnóstico Integral de Aprendizaje",
+        "input": "PDF",
+        "output": "Excel"
+    },
+    "context": {
+        "base_dir": "./backend/tests"
+    },
+    "pipeline": [
+        {
+            "step": "",
+            "params": {}
+        }
+    ]
+}</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
         <is>
           <t>PDF</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>EXCEL</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>2026-01-28 00:00:00</t>
         </is>
@@ -536,15 +635,82 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
+          <t>InitRun -&gt; LoadConfig -&gt; RequestUserFiles -&gt; RunExcelETL -&gt; EnrichWithContext -&gt; ExportConsolidatedExcel</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>{
+    "workflow_metadata": {
+        "name": "Proceso de prueba",
+        "description": "Testing pipeline",
+        "input": "EXCEL",
+        "output": "PDF"
+    },
+    "context": {
+        "base_dir": "tests"
+    },
+    "pipeline": [
+        {
+            "step": "InitRun",
+            "description": "",
+            "params": {
+                "inputs_dir": "tests/input_test/inputs/Lenguaje/inputs"
+            }
+        },
+        {
+            "step": "LoadConfig",
+            "description": "",
+            "params": {
+                "config_path": "./tests/config_dir/simce_estudiantes_lenguaje.json"
+            }
+        },
+        {
+            "step": "RequestUserFiles",
+            "description": "Cargue los archivos de puntajes asociado a los estudiantes",
+            "params": {
+                "file_specs": [
+                    {
+                        "id": "estudiantes",
+                        "label": "Archivos Excel de Estudiantes",
+                        "description": "Cargue los archivos Excel con los puntajes.",
+                        "multiple": true
+                    }
+                ]
+            }
+        },
+        {
+            "step": "RunExcelETL",
+            "description": "",
+            "params": {
+                "input_key": "estudiantes"
+            }
+        },
+        {
+            "step": "EnrichWithContext",
+            "description": "",
+            "params": {}
+        },
+        {
+            "step": "ExportConsolidatedExcel",
+            "description": "",
+            "params": {}
+        }
+    ]
+}</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
           <t>EXCEL</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>PDF</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>2026-02-04 13:20:30</t>
         </is>

</xml_diff>

<commit_message>
feat: EnrichWithUserInput feature para enriquecer df con información ingresada por el usuario
</commit_message>
<xml_diff>
--- a/data/database/pipelines.xlsx
+++ b/data/database/pipelines.xlsx
@@ -817,7 +817,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>InitRun -&gt; LoadConfigFromSpec -&gt; RequestUserFiles -&gt; RunExcelETL -&gt; EnrichWithContext -&gt; SaveToMetric</t>
+          <t>InitRun -&gt; LoadConfigFromSpec -&gt; RequestUserFiles -&gt; EnrichWithUserInput -&gt; RunExcelETL -&gt; EnrichWithContext</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -829,7 +829,9 @@
         "input": "EXCEL",
         "output": "PDF"
     },
-    "context": {},
+    "context": {
+        "base_dir": "./backend/tests"
+    },
     "pipeline": [
         {
             "step": "InitRun",
@@ -842,18 +844,18 @@
             "step": "LoadConfigFromSpec",
             "description": "",
             "params": {
-                "spec_id": 1
+                "spec_id": 2
             }
         },
         {
             "step": "RequestUserFiles",
-            "description": "",
+            "description": "Ingrese los archivos relacionados con las preguntas.",
             "params": {
                 "file_specs": [
                     {
-                        "id": "estudiantes",
-                        "label": "Archivos de estudiantes",
-                        "description": "Cargue los archivos de notas de estudiantes",
+                        "id": "preguntas",
+                        "label": "Archivos de preguntas",
+                        "description": "Cargue los archivos excel con la forma ReportePregunta",
                         "multiple": true,
                         "optional": false
                     }
@@ -861,28 +863,26 @@
             }
         },
         {
+            "step": "EnrichWithUserInput",
+            "description": "",
+            "params": {
+                "input_key": "preguntas"
+            }
+        },
+        {
             "step": "RunExcelETL",
             "description": "",
             "params": {
-                "input_key": "estudiantes",
-                "output_key": "df_estudiantes"
+                "input_key": "preguntas",
+                "output_key": "df_preguntas"
             }
         },
         {
             "step": "EnrichWithContext",
             "description": "",
             "params": {
-                "input_key": "df_estudiantes",
-                "output_key": "df_estudiantes"
-            }
-        },
-        {
-            "step": "SaveToMetric",
-            "description": "",
-            "params": {
-                "metric_id": 4,
-                "input_key": "df_estudiantes",
-                "clear_existing": false
+                "input_key": "df_preguntas",
+                "output_key": "df_preguntas"
             }
         }
     ]
@@ -901,7 +901,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-02-13 11:51:15</t>
+          <t>2026-02-13 16:48:25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
nuevo step para modificar valores de una columna
</commit_message>
<xml_diff>
--- a/data/database/pipelines.xlsx
+++ b/data/database/pipelines.xlsx
@@ -797,7 +797,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-02-12 18:02:13</t>
+          <t>2026-02-17 00:41:11</t>
         </is>
       </c>
     </row>
@@ -901,7 +901,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-02-13 16:48:25</t>
+          <t>2026-02-17 00:40:44</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Configuracion de métricas y pipelines
</commit_message>
<xml_diff>
--- a/data/database/pipelines.xlsx
+++ b/data/database/pipelines.xlsx
@@ -472,117 +472,20 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SIMCE Lenguaje</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Workflow SIMCE</t>
-        </is>
-      </c>
+          <t>[UT1] Cargar datos en métrica</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>InitRun -&gt; LoadConfig -&gt; DiscoverInputs -&gt; RunExcelETL -&gt; EnrichWithContext -&gt; ExportConsolidatedExcel</t>
+          <t>InitRun -&gt; RequestUserFiles -&gt; RunExcelETL -&gt; SaveToMetric</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
-        <is>
-          <t>{
-    "workflow_metadata": {
-        "name": "SIMCE Lenguaje",
-        "description": "Workflow SIMCE",
-        "input": "EXCEL",
-        "output": "PDF"
-    },
-    "context": {
-        "base_dir": "tests"
-    },
-    "pipeline": [
-        {
-            "step": "InitRun",
-            "params": {
-                "inputs_dir": "tests/input_test/inputs/Lenguaje/inputs"
-            }
-        },
-        {
-            "step": "LoadConfig",
-            "params": {
-                "config_path": "./tests/config_dir/simce_estudiantes_lenguaje.json"
-            }
-        },
-        {
-            "step": "DiscoverInputs",
-            "params": {
-                "rules": {
-                    "estudiantes": {
-                        "extension": ".xlsx",
-                        "contains": "Resultados"
-                    },
-                    "preguntas": {
-                        "extension": ".xlsx",
-                        "contains": "ReportePregunta"
-                    },
-                    "habilidades": {
-                        "extension": ".xlsx",
-                        "contains": "habilidades"
-                    }
-                }
-            }
-        },
-        {
-            "step": "RunExcelETL",
-            "params": {
-                "input_key": "estudiantes"
-            }
-        },
-        {
-            "step": "EnrichWithContext",
-            "params": {}
-        },
-        {
-            "step": "ExportConsolidatedExcel",
-            "params": {}
-        }
-    ]
-}</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>EXCEL</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>2026-01-31 13:28:43</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>11</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>[UT1] Cargar datos en métrica</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>InitRun -&gt; RequestUserFiles -&gt; RunExcelETL -&gt; SaveToMetric</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
         <is>
           <t>{
     "pipeline_metadata": {
@@ -636,42 +539,42 @@
 }</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>EXCEL</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>DB</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>2026-02-17 00:41:11</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="n">
+    <row r="3">
+      <c r="A3" t="n">
         <v>12</v>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>SIMCE Lenguaje 2</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Workflow SIMCE</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>InitRun -&gt; LoadConfigFromSpec -&gt; RequestUserFiles -&gt; EnrichWithUserInput -&gt; RunExcelETL -&gt; EnrichWithContext</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>{
     "pipeline_metadata": {
@@ -740,6 +643,163 @@
 }</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>EXCEL</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-02-17 00:40:44</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>13</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>SIMCE Lenguaje</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>InitRun -&gt; LoadConfigFromSpec -&gt; RequestUserFiles -&gt; RunExcelETL -&gt; EnrichWithContext -&gt; LoadConfigFromSpec -&gt; RequestUserFiles -&gt; EnrichWithUserInput -&gt; RunExcelETL -&gt; EnrichWithContext -&gt; SaveToMetric -&gt; SaveToMetric</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>{
+    "pipeline_metadata": {
+        "name": "SIMCE Lenguaje",
+        "description": "",
+        "input": "EXCEL",
+        "output": "IMG"
+    },
+    "context": {
+        "evaluation": "simce_lenguaje"
+    },
+    "pipeline": [
+        {
+            "step": "InitRun",
+            "description": "",
+            "params": {
+                "evaluation": "simce_lenguaje",
+                "base_dir": "./tests"
+            }
+        },
+        {
+            "step": "LoadConfigFromSpec",
+            "description": "",
+            "params": {
+                "spec_id": 1
+            }
+        },
+        {
+            "step": "RequestUserFiles",
+            "description": "Ingrese los archivos relacionados a puntaje de la evaluación por estudiante",
+            "params": {
+                "file_specs": [
+                    {
+                        "id": "estudiantes",
+                        "label": "Resultados Estudiantes",
+                        "description": "",
+                        "multiple": true,
+                        "optional": false
+                    }
+                ]
+            }
+        },
+        {
+            "step": "RunExcelETL",
+            "description": "",
+            "params": {
+                "input_key": "estudiantes",
+                "output_key": "estudiantes"
+            }
+        },
+        {
+            "step": "EnrichWithContext",
+            "description": "",
+            "params": {
+                "input_key": "estudiantes",
+                "output_key": "estudiantes"
+            }
+        },
+        {
+            "step": "LoadConfigFromSpec",
+            "description": "",
+            "params": {
+                "spec_id": 2
+            }
+        },
+        {
+            "step": "RequestUserFiles",
+            "description": "Ingrese los archivos de resultados por preguntas",
+            "params": {
+                "file_specs": [
+                    {
+                        "id": "preguntas",
+                        "label": "Resultados por preguntas",
+                        "description": "",
+                        "multiple": true,
+                        "optional": false
+                    }
+                ]
+            }
+        },
+        {
+            "step": "EnrichWithUserInput",
+            "description": "",
+            "params": {
+                "input_key": "preguntas"
+            }
+        },
+        {
+            "step": "RunExcelETL",
+            "description": "",
+            "params": {
+                "input_key": "preguntas",
+                "output_key": "preguntas"
+            }
+        },
+        {
+            "step": "EnrichWithContext",
+            "description": "",
+            "params": {
+                "input_key": "preguntas",
+                "output_key": "preguntas"
+            }
+        },
+        {
+            "step": "SaveToMetric",
+            "description": "",
+            "params": {
+                "metric_id": 4,
+                "input_key": "estudiantes",
+                "clear_existing": false
+            }
+        },
+        {
+            "step": "SaveToMetric",
+            "description": "PENDIENTE: Falta agregar la métrica de preguntas",
+            "params": {
+                "metric_id": 5,
+                "input_key": "preguntas",
+                "clear_existing": false
+            }
+        }
+    ]
+}</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
           <t>EXCEL</t>
@@ -747,14 +807,10 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>2026-02-17 00:40:44</t>
-        </is>
-      </c>
+          <t>IMG</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Se crean pasos para crear tablas, se configuran pipelines de testing
</commit_message>
<xml_diff>
--- a/data/database/pipelines.xlsx
+++ b/data/database/pipelines.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -557,281 +557,24 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>SIMCE Lenguaje 2</t>
+          <t>SIMCE Lenguaje (IA)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Workflow SIMCE</t>
+          <t>Clon automatizado de SIMCE Lenguaje con modificación de Curso, join de habilidades y guardado en métricas.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>InitRun -&gt; LoadConfigFromSpec -&gt; RequestUserFiles -&gt; EnrichWithUserInput -&gt; RunExcelETL -&gt; EnrichWithContext</t>
+          <t>InitRun -&gt; LoadConfigFromSpec -&gt; RequestUserFiles -&gt; RunExcelETL -&gt; ModifyColumnValues -&gt; EnrichWithContext -&gt; LoadConfigFromSpec -&gt; RequestUserFiles -&gt; EnrichWithUserInput -&gt; RunExcelETL -&gt; EnrichWithContext -&gt; RequestUserFiles -&gt; LoadConfigFromSpec -&gt; RunExcelETL -&gt; EnrichWithLookup -&gt; SaveToMetric -&gt; SaveToMetric</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
-        <is>
-          <t>{
-    "pipeline_metadata": {
-        "name": "SIMCE Lenguaje 2",
-        "description": "Workflow SIMCE",
-        "input": "EXCEL",
-        "output": "PDF"
-    },
-    "context": {
-        "base_dir": "./backend/tests"
-    },
-    "pipeline": [
-        {
-            "step": "InitRun",
-            "description": "",
-            "params": {
-                "inputs_dir": "tests/input_test/inputs/Lenguaje/inputs"
-            }
-        },
-        {
-            "step": "LoadConfigFromSpec",
-            "description": "",
-            "params": {
-                "spec_id": 2
-            }
-        },
-        {
-            "step": "RequestUserFiles",
-            "description": "Ingrese los archivos relacionados con las preguntas.",
-            "params": {
-                "file_specs": [
-                    {
-                        "id": "preguntas",
-                        "label": "Archivos de preguntas",
-                        "description": "Cargue los archivos excel con la forma ReportePregunta",
-                        "multiple": true,
-                        "optional": false
-                    }
-                ]
-            }
-        },
-        {
-            "step": "EnrichWithUserInput",
-            "description": "",
-            "params": {
-                "input_key": "preguntas"
-            }
-        },
-        {
-            "step": "RunExcelETL",
-            "description": "",
-            "params": {
-                "input_key": "preguntas",
-                "output_key": "df_preguntas"
-            }
-        },
-        {
-            "step": "EnrichWithContext",
-            "description": "",
-            "params": {
-                "input_key": "df_preguntas",
-                "output_key": "df_preguntas"
-            }
-        }
-    ]
-}</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>EXCEL</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>2026-02-17 00:40:44</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>13</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>SIMCE Lenguaje</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>InitRun -&gt; LoadConfigFromSpec -&gt; RequestUserFiles -&gt; RunExcelETL -&gt; EnrichWithContext -&gt; LoadConfigFromSpec -&gt; RequestUserFiles -&gt; EnrichWithUserInput -&gt; RunExcelETL -&gt; EnrichWithContext -&gt; SaveToMetric -&gt; SaveToMetric</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>{
-    "pipeline_metadata": {
-        "name": "SIMCE Lenguaje",
-        "description": "",
-        "input": "EXCEL",
-        "output": "IMG"
-    },
-    "context": {
-        "evaluation": "simce_lenguaje"
-    },
-    "pipeline": [
-        {
-            "step": "InitRun",
-            "description": "",
-            "params": {
-                "evaluation": "simce_lenguaje",
-                "base_dir": "./tests"
-            }
-        },
-        {
-            "step": "LoadConfigFromSpec",
-            "description": "",
-            "params": {
-                "spec_id": 1
-            }
-        },
-        {
-            "step": "RequestUserFiles",
-            "description": "Ingrese los archivos relacionados a puntaje de la evaluación por estudiante",
-            "params": {
-                "file_specs": [
-                    {
-                        "id": "estudiantes",
-                        "label": "Resultados Estudiantes",
-                        "description": "",
-                        "multiple": true,
-                        "optional": false
-                    }
-                ]
-            }
-        },
-        {
-            "step": "RunExcelETL",
-            "description": "",
-            "params": {
-                "input_key": "estudiantes",
-                "output_key": "estudiantes"
-            }
-        },
-        {
-            "step": "EnrichWithContext",
-            "description": "",
-            "params": {
-                "input_key": "estudiantes",
-                "output_key": "estudiantes"
-            }
-        },
-        {
-            "step": "LoadConfigFromSpec",
-            "description": "",
-            "params": {
-                "spec_id": 2
-            }
-        },
-        {
-            "step": "RequestUserFiles",
-            "description": "Ingrese los archivos de resultados por preguntas",
-            "params": {
-                "file_specs": [
-                    {
-                        "id": "preguntas",
-                        "label": "Resultados por preguntas",
-                        "description": "",
-                        "multiple": true,
-                        "optional": false
-                    }
-                ]
-            }
-        },
-        {
-            "step": "EnrichWithUserInput",
-            "description": "",
-            "params": {
-                "input_key": "preguntas"
-            }
-        },
-        {
-            "step": "RunExcelETL",
-            "description": "",
-            "params": {
-                "input_key": "preguntas",
-                "output_key": "preguntas"
-            }
-        },
-        {
-            "step": "EnrichWithContext",
-            "description": "",
-            "params": {
-                "input_key": "preguntas",
-                "output_key": "preguntas"
-            }
-        },
-        {
-            "step": "SaveToMetric",
-            "description": "",
-            "params": {
-                "metric_id": 4,
-                "input_key": "estudiantes",
-                "clear_existing": false
-            }
-        },
-        {
-            "step": "SaveToMetric",
-            "description": "PENDIENTE: Falta agregar la métrica de preguntas",
-            "params": {
-                "metric_id": 5,
-                "input_key": "preguntas",
-                "clear_existing": false
-            }
-        }
-    ]
-}</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>EXCEL</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>IMG</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>14</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>SIMCE Lenguaje (IA)</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Clon automatizado de SIMCE Lenguaje con modificación de Curso, join de habilidades y guardado en métricas.</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>InitRun -&gt; LoadConfigFromSpec -&gt; RequestUserFiles -&gt; RunExcelETL -&gt; ModifyColumnValues -&gt; EnrichWithContext -&gt; LoadConfigFromSpec -&gt; RequestUserFiles -&gt; EnrichWithUserInput -&gt; RunExcelETL -&gt; EnrichWithContext -&gt; RequestUserFiles -&gt; LoadConfigFromSpec -&gt; RunExcelETL -&gt; EnrichWithLookup -&gt; SaveToMetric -&gt; SaveToMetric</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
         <is>
           <t>{
     "pipeline_metadata": {
@@ -1027,144 +770,326 @@
 }</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>EXCEL</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>DB</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>2026-03-03 21:47:36</t>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-03-05 18:09:24</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>15</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>DEBUG Habilidades</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Pipeline de debug para aislar RequestUserFiles + RunExcelETL de habilidades</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>InitRun -&gt; RequestUserFiles -&gt; RunExcelETL -&gt; LoadConfigFromSpec -&gt; RequestUserFiles -&gt; RunExcelETL -&gt; EnrichWithLookup</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="n">
+        <v>16</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>SIMCE Lenguaje - Gráficos</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Carga métricas SIMCE y genera todos los gráficos de rendimiento</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>InitRun -&gt; LoadMetricToDF -&gt; LoadMetricToDF -&gt; LoadMetricToDF -&gt; GenerateGraphics</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>{
+    "context": {
+        "evaluation": "simce_lenguaje"
+    },
+    "pipeline": [
+        {
+            "step": "InitRun",
+            "params": {
+                "evaluation": "simce_lenguaje"
+            }
+        },
+        {
+            "step": "LoadMetricToDF",
+            "params": {
+                "metric_id": 4,
+                "output_key": "df_estudiantes"
+            }
+        },
+        {
+            "step": "LoadMetricToDF",
+            "params": {
+                "metric_id": 4,
+                "output_key": "df_estudiantes_prueba",
+                "filters": {
+                    "Numero_Prueba": 5
+                }
+            }
+        },
+        {
+            "step": "LoadMetricToDF",
+            "params": {
+                "metric_id": 5,
+                "output_key": "df_preguntas"
+            }
+        },
+        {
+            "step": "GenerateGraphics",
+            "params": {
+                "charts_schema": [
+                    {
+                        "id": "rendimiento_promedio_curso",
+                        "title": "Rendimiento Promedio por Curso",
+                        "category": "resumen",
+                        "type": "grafico_barras_promedio_por",
+                        "input_key": "df_estudiantes_prueba",
+                        "output_filename": "rendimiento_promedio_por_curso.png",
+                        "params": {
+                            "columna_valor": "Rend",
+                            "agrupar_por": "Curso",
+                            "titulo": "Rendimiento Promedio por Curso",
+                            "ylabel": "Rendimiento (%)"
+                        }
+                    },
+                    {
+                        "id": "distribucion_simce_curso",
+                        "title": "Distribución de Puntaje SIMCE por Curso",
+                        "category": "resumen",
+                        "type": "boxplot_valor_por_curso",
+                        "input_key": "df_estudiantes_prueba",
+                        "output_filename": "distribucion_puntaje_simce_por_curso.png",
+                        "params": {
+                            "columna_valor": "SIMCE",
+                            "agrupar_por": "Curso",
+                            "titulo_grafico": "Distribución de Puntaje SIMCE por Curso",
+                            "ylabel": "Puntaje SIMCE",
+                            "formato": "number"
+                        }
+                    },
+                    {
+                        "id": "alumnos_por_nivel_curso",
+                        "title": "Alumnos por Nivel de Logro y Curso",
+                        "category": "resumen",
+                        "type": "alumnos_por_nivel_cualitativo",
+                        "input_key": "df_estudiantes_prueba",
+                        "output_filename": "alumnos_por_nivel.png",
+                        "params": {
+                            "columna_nivel": "Logro",
+                            "agrupar_por": "Curso",
+                            "titulo_grafico": "Cantidad de Alumnos por Nivel de Logro y Curso",
+                            "titulo_leyenda": "Nivel de Logro",
+                            "ylabel": "Cantidad de Alumnos"
+                        }
+                    },
+                    {
+                        "id": "evolucion_logro_mes",
+                        "title": "Evolución del Logro Promedio por Curso y Mes",
+                        "category": "evolucion",
+                        "type": "valor_promedio_agrupado_por",
+                        "input_key": "df_estudiantes",
+                        "output_filename": "evolucion_logro_promedio_por_curso_y_mes.png",
+                        "params": {
+                            "columna_valor": "Rend",
+                            "agrupar_principal_por": "Curso",
+                            "agrupar_secundario_por": "Mes",
+                            "titulo_grafico": "Evolución del Logro Promedio por Curso y Mes",
+                            "titulo_leyenda": "Mes",
+                            "y_lims": [
+                                0,
+                                1
+                            ],
+                            "formato": "percent"
+                        }
+                    },
+                    {
+                        "id": "evolucion_simce_mes",
+                        "title": "Evolución del SIMCE Promedio por Curso y Mes",
+                        "category": "evolucion",
+                        "type": "valor_promedio_agrupado_por",
+                        "input_key": "df_estudiantes",
+                        "output_filename": "evolucion_simce_promedio_por_curso_y_mes.png",
+                        "params": {
+                            "columna_valor": "SIMCE",
+                            "agrupar_principal_por": "Curso",
+                            "agrupar_secundario_por": "Mes",
+                            "titulo_grafico": "Evolución del SIMCE Promedio por Curso y Mes",
+                            "titulo_leyenda": "Mes",
+                            "formato": "number"
+                        }
+                    },
+                    {
+                        "id": "evolucion_alumnos_nivel_mes",
+                        "title": "Evolución de Alumnos por Nivel y Mes",
+                        "category": "evolucion",
+                        "type": "alumnos_por_nivel_curso_y_mes",
+                        "input_key": "df_estudiantes",
+                        "output_filename": "evolucion_alumnos_por_nivel.png",
+                        "params": {
+                            "columna_nivel": "Logro",
+                            "titulo_grafico": "",
+                            "titulo_leyenda": "Nivel de Logro",
+                            "ylabel": "Cantidad de Alumnos"
+                        }
+                    },
+                    {
+                        "id": "logro_por_habilidad",
+                        "title": "Logro Promedio por Habilidad",
+                        "category": "preguntas",
+                        "type": "valor_promedio_agrupado_por",
+                        "input_key": "df_preguntas",
+                        "output_filename": "logro_promedio_por_habilidad.png",
+                        "params": {
+                            "columna_valor": "Logro",
+                            "agrupar_principal_por": "Curso",
+                            "agrupar_secundario_por": "Habilidad",
+                            "titulo_grafico": "Logro Promedio por Habilidad",
+                            "titulo_leyenda": "Habilidad",
+                            "formato": "percent"
+                        }
+                    },
+                    {
+                        "id": "logro_por_eje",
+                        "title": "Logro Promedio por Eje Temático",
+                        "category": "preguntas",
+                        "type": "valor_promedio_agrupado_por",
+                        "input_key": "df_preguntas",
+                        "output_filename": "logro_promedio_por_eje.png",
+                        "params": {
+                            "columna_valor": "Logro",
+                            "agrupar_principal_por": "Curso",
+                            "agrupar_secundario_por": "Eje temático",
+                            "titulo_grafico": "Logro Promedio por Eje Temático",
+                            "titulo_leyenda": "Eje Temático",
+                            "formato": "percent"
+                        }
+                    }
+                ]
+            }
+        }
+    ],
+    "pipeline_metadata": {
+        "name": "SIMCE Lenguaje - Gráficos",
+        "description": "Carga métricas SIMCE y genera todos los gráficos de rendimiento",
+        "input": "DB",
+        "output": "IMG"
+    }
+}</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>IMG</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-03-05 18:09:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>17</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>SIMCE Lenguaje - Tablas</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Carga métricas SIMCE y genera tablas de logro y estadísticas</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>InitRun -&gt; LoadMetricToDF -&gt; LoadMetricToDF -&gt; LoadMetricToDF -&gt; LoadConfigFromSpec -&gt; GenerateTables</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
         <is>
           <t>{
     "pipeline_metadata": {
-        "name": "DEBUG Habilidades",
-        "description": "Pipeline de debug para aislar RequestUserFiles + RunExcelETL de habilidades",
-        "input": "EXCEL",
-        "output": "DB"
+        "name": "SIMCE Lenguaje - Tablas",
+        "description": "Carga métricas SIMCE y genera tablas de logro y estadísticas",
+        "input": "DB",
+        "output": "EXCEL"
     },
-    "context": {},
+    "context": {
+        "evaluation": "simce_lenguaje"
+    },
     "pipeline": [
         {
             "step": "InitRun",
-            "description": "",
+            "params": {
+                "evaluation": "simce_lenguaje"
+            }
+        },
+        {
+            "step": "LoadMetricToDF",
+            "params": {
+                "metric_id": 4,
+                "output_key": "df_estudiantes"
+            }
+        },
+        {
+            "step": "LoadMetricToDF",
+            "params": {
+                "metric_id": 4,
+                "output_key": "df_estudiantes_prueba",
+                "filters": {
+                    "Numero_Prueba": 5
+                }
+            }
+        },
+        {
+            "step": "LoadMetricToDF",
+            "params": {
+                "metric_id": 5,
+                "output_key": "df_preguntas"
+            }
+        },
+        {
+            "step": "LoadConfigFromSpec",
+            "params": {
+                "spec_id": 4
+            }
+        },
+        {
+            "step": "GenerateTables",
             "params": {}
-        },
-        {
-            "step": "RequestUserFiles",
-            "description": "Ingrese el archivo de habilidades por pregunta",
-            "params": {
-                "file_specs": [
-                    {
-                        "id": "habilidades",
-                        "label": "Archivo de habilidades",
-                        "description": "Archivo Excel con columnas N° y Habilidad por pregunta",
-                        "multiple": false,
-                        "optional": false
-                    }
-                ]
-            }
-        },
-        {
-            "step": "RunExcelETL",
-            "description": "",
-            "params": {
-                "input_key": "habilidades",
-                "output_key": "habilidades"
-            }
-        },
-        {
-            "step": "LoadConfigFromSpec",
-            "description": "",
-            "params": {
-                "spec_id": 2,
-                "input_key": "preguntas"
-            }
-        },
-        {
-            "step": "RequestUserFiles",
-            "description": "Ingrese archivos de preguntas para probar el join",
-            "params": {
-                "file_specs": [
-                    {
-                        "id": "preguntas",
-                        "label": "Resultados por preguntas",
-                        "description": "",
-                        "multiple": true,
-                        "optional": false
-                    }
-                ]
-            }
-        },
-        {
-            "step": "RunExcelETL",
-            "description": "",
-            "params": {
-                "input_key": "preguntas",
-                "output_key": "preguntas"
-            }
-        },
-        {
-            "step": "EnrichWithLookup",
-            "description": "Join left entre preguntas y habilidades por Pregunta &lt;-&gt; N°",
-            "params": {
-                "input_key": "preguntas",
-                "lookup_key": "habilidades",
-                "left_on": "Pregunta",
-                "right_on": "N°",
-                "columns": [
-                    "N°",
-                    "Habilidad"
-                ],
-                "output_key": "preguntas",
-                "how": "left"
-            }
         }
     ]
 }</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
         <is>
           <t>EXCEL</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>DB</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>2026-03-03 20:25:51</t>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-03-05 18:31:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: enable management of chart and table schemas for report specifications
</commit_message>
<xml_diff>
--- a/data/database/pipelines.xlsx
+++ b/data/database/pipelines.xlsx
@@ -802,7 +802,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>InitRun -&gt; LoadMetricToDF -&gt; LoadMetricToDF -&gt; LoadMetricToDF -&gt; GenerateGraphics</t>
+          <t>InitRun -&gt; LoadMetricToDF -&gt; LoadMetricToDF -&gt; LoadMetricToDF -&gt; LoadConfigFromSpec -&gt; LoadConfigFromSpec -&gt; GenerateGraphics</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -843,142 +843,25 @@
             }
         },
         {
+            "step": "LoadConfigFromSpec",
+            "params": {
+                "spec_id": 5
+            }
+        },
+        {
+            "step": "LoadConfigFromSpec",
+            "params": {
+                "spec_id": 5
+            }
+        },
+        {
             "step": "GenerateGraphics",
-            "params": {
-                "charts_schema": [
-                    {
-                        "id": "rendimiento_promedio_curso",
-                        "title": "Rendimiento Promedio por Curso",
-                        "category": "resumen",
-                        "type": "grafico_barras_promedio_por",
-                        "input_key": "df_estudiantes_prueba",
-                        "output_filename": "rendimiento_promedio_por_curso.png",
-                        "params": {
-                            "columna_valor": "Rend",
-                            "agrupar_por": "Curso",
-                            "titulo": "Rendimiento Promedio por Curso",
-                            "ylabel": "Rendimiento (%)"
-                        }
-                    },
-                    {
-                        "id": "distribucion_simce_curso",
-                        "title": "Distribución de Puntaje SIMCE por Curso",
-                        "category": "resumen",
-                        "type": "boxplot_valor_por_curso",
-                        "input_key": "df_estudiantes_prueba",
-                        "output_filename": "distribucion_puntaje_simce_por_curso.png",
-                        "params": {
-                            "columna_valor": "SIMCE",
-                            "agrupar_por": "Curso",
-                            "titulo_grafico": "Distribución de Puntaje SIMCE por Curso",
-                            "ylabel": "Puntaje SIMCE",
-                            "formato": "number"
-                        }
-                    },
-                    {
-                        "id": "alumnos_por_nivel_curso",
-                        "title": "Alumnos por Nivel de Logro y Curso",
-                        "category": "resumen",
-                        "type": "alumnos_por_nivel_cualitativo",
-                        "input_key": "df_estudiantes_prueba",
-                        "output_filename": "alumnos_por_nivel.png",
-                        "params": {
-                            "columna_nivel": "Logro",
-                            "agrupar_por": "Curso",
-                            "titulo_grafico": "Cantidad de Alumnos por Nivel de Logro y Curso",
-                            "titulo_leyenda": "Nivel de Logro",
-                            "ylabel": "Cantidad de Alumnos"
-                        }
-                    },
-                    {
-                        "id": "evolucion_logro_mes",
-                        "title": "Evolución del Logro Promedio por Curso y Mes",
-                        "category": "evolucion",
-                        "type": "valor_promedio_agrupado_por",
-                        "input_key": "df_estudiantes",
-                        "output_filename": "evolucion_logro_promedio_por_curso_y_mes.png",
-                        "params": {
-                            "columna_valor": "Rend",
-                            "agrupar_principal_por": "Curso",
-                            "agrupar_secundario_por": "Mes",
-                            "titulo_grafico": "Evolución del Logro Promedio por Curso y Mes",
-                            "titulo_leyenda": "Mes",
-                            "y_lims": [
-                                0,
-                                1
-                            ],
-                            "formato": "percent"
-                        }
-                    },
-                    {
-                        "id": "evolucion_simce_mes",
-                        "title": "Evolución del SIMCE Promedio por Curso y Mes",
-                        "category": "evolucion",
-                        "type": "valor_promedio_agrupado_por",
-                        "input_key": "df_estudiantes",
-                        "output_filename": "evolucion_simce_promedio_por_curso_y_mes.png",
-                        "params": {
-                            "columna_valor": "SIMCE",
-                            "agrupar_principal_por": "Curso",
-                            "agrupar_secundario_por": "Mes",
-                            "titulo_grafico": "Evolución del SIMCE Promedio por Curso y Mes",
-                            "titulo_leyenda": "Mes",
-                            "formato": "number"
-                        }
-                    },
-                    {
-                        "id": "evolucion_alumnos_nivel_mes",
-                        "title": "Evolución de Alumnos por Nivel y Mes",
-                        "category": "evolucion",
-                        "type": "alumnos_por_nivel_curso_y_mes",
-                        "input_key": "df_estudiantes",
-                        "output_filename": "evolucion_alumnos_por_nivel.png",
-                        "params": {
-                            "columna_nivel": "Logro",
-                            "titulo_grafico": "",
-                            "titulo_leyenda": "Nivel de Logro",
-                            "ylabel": "Cantidad de Alumnos"
-                        }
-                    },
-                    {
-                        "id": "logro_por_habilidad",
-                        "title": "Logro Promedio por Habilidad",
-                        "category": "preguntas",
-                        "type": "valor_promedio_agrupado_por",
-                        "input_key": "df_preguntas",
-                        "output_filename": "logro_promedio_por_habilidad.png",
-                        "params": {
-                            "columna_valor": "Logro",
-                            "agrupar_principal_por": "Curso",
-                            "agrupar_secundario_por": "Habilidad",
-                            "titulo_grafico": "Logro Promedio por Habilidad",
-                            "titulo_leyenda": "Habilidad",
-                            "formato": "percent"
-                        }
-                    },
-                    {
-                        "id": "logro_por_eje",
-                        "title": "Logro Promedio por Eje Temático",
-                        "category": "preguntas",
-                        "type": "valor_promedio_agrupado_por",
-                        "input_key": "df_preguntas",
-                        "output_filename": "logro_promedio_por_eje.png",
-                        "params": {
-                            "columna_valor": "Logro",
-                            "agrupar_principal_por": "Curso",
-                            "agrupar_secundario_por": "Eje temático",
-                            "titulo_grafico": "Logro Promedio por Eje Temático",
-                            "titulo_leyenda": "Eje Temático",
-                            "formato": "percent"
-                        }
-                    }
-                ]
-            }
+            "params": {}
         }
     ],
     "pipeline_metadata": {
-        "name": "SIMCE Lenguaje - Gráficos",
-        "description": "Carga métricas SIMCE y genera todos los gráficos de rendimiento",
+        "name": "SIMCE Lenguaje - Gr\u00e1ficos",
+        "description": "Carga m\u00e9tricas SIMCE y genera todos los gr\u00e1ficos de rendimiento",
         "input": "DB",
         "output": "IMG"
     }

</xml_diff>

<commit_message>
fixed pipeline with spec loadings
</commit_message>
<xml_diff>
--- a/data/database/pipelines.xlsx
+++ b/data/database/pipelines.xlsx
@@ -802,7 +802,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>InitRun -&gt; LoadMetricToDF -&gt; LoadMetricToDF -&gt; LoadMetricToDF -&gt; LoadConfigFromSpec -&gt; LoadConfigFromSpec -&gt; GenerateGraphics</t>
+          <t>InitRun -&gt; LoadMetricToDF -&gt; LoadMetricToDF -&gt; LoadMetricToDF -&gt; LoadConfigFromSpec -&gt; GenerateGraphics</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -840,12 +840,6 @@
             "params": {
                 "metric_id": 5,
                 "output_key": "df_preguntas"
-            }
-        },
-        {
-            "step": "LoadConfigFromSpec",
-            "params": {
-                "spec_id": 5
             }
         },
         {

</xml_diff>

<commit_message>
Funcionalidad: Botón mostrar/ocultar procesos
</commit_message>
<xml_diff>
--- a/data/database/pipelines.xlsx
+++ b/data/database/pipelines.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,11 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>last_run</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>hidden</t>
         </is>
       </c>
     </row>
@@ -553,6 +558,9 @@
         <is>
           <t>2026-02-17 00:41:11</t>
         </is>
+      </c>
+      <c r="I2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -830,6 +838,9 @@
           <t>2026-03-10 18:08:59</t>
         </is>
       </c>
+      <c r="I3" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -922,6 +933,9 @@
           <t>2026-03-05 18:09:32</t>
         </is>
       </c>
+      <c r="I4" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -1014,6 +1028,9 @@
           <t>2026-03-05 18:31:00</t>
         </is>
       </c>
+      <c r="I5" t="b">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix: migrate backend to package structure and add JWT auth to all API calls
- Add backend/__init__.py and backend/routers/__init__.py to fix module resolution
- Fix api.py imports to use backend.routers prefix and correct uvicorn path
- Add fetchAuth to all frontend pages/components that were using plain fetch
- Fix SuperAdmin.jsx await inside setState callback
- Fix Execution.jsx Array.isArray guard for pipelines response
- Rewrite run_software.bat to start PostgreSQL Windows service
- Remove restart_backend.bat and run_software.sh
- Add DB diagnostic and re-migration scripts
- Ignore .claude/worktrees/ in .gitignore

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/database/pipelines.xlsx
+++ b/data/database/pipelines.xlsx
@@ -1184,8 +1184,8 @@
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
-      <c r="I8" t="n">
-        <v>0</v>
+      <c r="I8" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>